<commit_message>
fix(w01): restore original interview export filenames
</commit_message>
<xml_diff>
--- a/artifacts/w01/product_fit_gap.xlsx
+++ b/artifacts/w01/product_fit_gap.xlsx
@@ -94,6 +94,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF24364B"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>三个月已确认是沈总</t>
     </r>
     <r>
@@ -289,6 +295,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF24364B"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>"</t>
     </r>
     <r>
@@ -421,6 +433,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF24364B"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>"</t>
     </r>
     <r>
@@ -574,6 +592,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF24364B"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>形式上沈总倾向名单</t>
     </r>
     <r>
@@ -801,7 +825,7 @@
     <t>沈总不只是需要一个功能列表一个一次性的产品，关心的是产品能达到什么样的效果</t>
   </si>
   <si>
-    <t>artifacts/w01/evidence/interviews/01-沈总-20261021-public.json</t>
+    <t>artifacts/w01/evidence/interviews/W1-interview-c2df6ffe-7cef-5250-92ea-9426236244f7-public.json</t>
   </si>
   <si>
     <t>MSG-00659</t>
@@ -1478,7 +1502,7 @@
     </border>
   </borders>
   <cellStyleXfs count="50">
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1627,7 +1651,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1663,9 +1687,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2293,7 +2314,7 @@
       <c r="E11" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="9" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2313,7 +2334,7 @@
       <c r="E12" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="9" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2333,7 +2354,7 @@
       <c r="E13" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="13" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3345,7 +3366,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" ht="44" customHeight="1" spans="1:4">
+    <row r="20" ht="51" spans="1:4">
       <c r="A20" s="9" t="s">
         <v>22</v>
       </c>
@@ -3415,7 +3436,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="25" ht="44" customHeight="1" spans="1:4">
+    <row r="25" ht="51" spans="1:4">
       <c r="A25" s="9" t="s">
         <v>26</v>
       </c>
@@ -3471,7 +3492,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" ht="44" customHeight="1" spans="1:4">
+    <row r="29" ht="51" spans="1:4">
       <c r="A29" s="9" t="s">
         <v>30</v>
       </c>

</xml_diff>